<commit_message>
feat: initialize Web and WebApi projects with Bootstrap assets and base configuration
</commit_message>
<xml_diff>
--- a/docs/Tablas Movimientos.xlsx
+++ b/docs/Tablas Movimientos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Proyectos\FinanKore\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Proyectos\FinanKore\Financore\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148F003E-DA48-4BE7-B529-2C66090A7581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A83AB2-AB36-4412-B771-312078A3176A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{57ED79E0-A070-4370-834F-0964443A1EE9}"/>
+    <workbookView xWindow="-2544" yWindow="2472" windowWidth="17280" windowHeight="8880" xr2:uid="{57ED79E0-A070-4370-834F-0964443A1EE9}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>